<commit_message>
fix: refine capture blocks and parcel table rendering
Crop contract/BACEN captures to target sections, expand long calculation block ranges to avoid truncation, and hide helper cell C5 in the template. Also bump to v0.6.1 and keep dynamic parcel formulas plus regression checks for table rows.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/templates/Calculo.xlsx
+++ b/templates/Calculo.xlsx
@@ -186,7 +186,7 @@
     <numFmt numFmtId="175" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="176" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -339,6 +339,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -787,7 +795,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="410">
+  <cellXfs count="411">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1948,6 +1956,9 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="175" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="23">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4691,11 +4702,7 @@
       <c r="CC4" s="254" t="n"/>
     </row>
     <row r="5" ht="6" customHeight="1" s="250">
-      <c r="C5" s="256" t="inlineStr">
-        <is>
-          <t>Data do 1º vencimento:</t>
-        </is>
-      </c>
+      <c r="C5" s="410" t="inlineStr"/>
       <c r="D5" s="257">
         <f>DADOS!$B$4</f>
         <v/>
@@ -14625,11 +14632,12 @@
       <c r="CI131" s="316" t="n"/>
     </row>
     <row r="132" ht="15.75" customHeight="1" s="250">
-      <c r="C132" s="392" t="n">
-        <v>1</v>
+      <c r="C132" s="392">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D132" s="393">
-        <f>IF(C132&lt;=$I$15, $D$5, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E132" s="272" t="n"/>
@@ -14642,7 +14650,7 @@
       <c r="L132" s="272" t="n"/>
       <c r="M132" s="273" t="n"/>
       <c r="N132" s="274">
-        <f>IF(C132&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O132" s="272" t="n"/>
@@ -14712,7 +14720,7 @@
       <c r="BN132" s="272" t="n"/>
       <c r="BO132" s="273" t="n"/>
       <c r="BP132" s="274">
-        <f>N132</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ132" s="272" t="n"/>
@@ -14731,11 +14739,12 @@
       <c r="CI132" s="316" t="n"/>
     </row>
     <row r="133" ht="15.75" customHeight="1" s="250">
-      <c r="C133" s="282" t="n">
-        <v>2</v>
+      <c r="C133" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D133" s="393">
-        <f>IF(C133&lt;=$I$15, EDATE($D$5, C133-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E133" s="272" t="n"/>
@@ -14748,7 +14757,7 @@
       <c r="L133" s="272" t="n"/>
       <c r="M133" s="273" t="n"/>
       <c r="N133" s="394">
-        <f>IF(C133&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O133" s="279" t="n"/>
@@ -14818,7 +14827,7 @@
       <c r="BN133" s="279" t="n"/>
       <c r="BO133" s="280" t="n"/>
       <c r="BP133" s="394">
-        <f>BP132</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ133" s="279" t="n"/>
@@ -14837,11 +14846,12 @@
       <c r="CI133" s="316" t="n"/>
     </row>
     <row r="134" ht="15.75" customHeight="1" s="250">
-      <c r="C134" s="282" t="n">
-        <v>3</v>
+      <c r="C134" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D134" s="393">
-        <f>IF(C134&lt;=$I$15, EDATE($D$5, C134-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E134" s="272" t="n"/>
@@ -14854,7 +14864,7 @@
       <c r="L134" s="272" t="n"/>
       <c r="M134" s="273" t="n"/>
       <c r="N134" s="394">
-        <f>IF(C134&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O134" s="279" t="n"/>
@@ -14924,7 +14934,7 @@
       <c r="BN134" s="279" t="n"/>
       <c r="BO134" s="280" t="n"/>
       <c r="BP134" s="394">
-        <f>BP133</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ134" s="279" t="n"/>
@@ -14943,11 +14953,12 @@
       <c r="CI134" s="316" t="n"/>
     </row>
     <row r="135" ht="15.75" customHeight="1" s="250">
-      <c r="C135" s="282" t="n">
-        <v>4</v>
+      <c r="C135" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D135" s="393">
-        <f>IF(C135&lt;=$I$15, EDATE($D$5, C135-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E135" s="272" t="n"/>
@@ -14960,7 +14971,7 @@
       <c r="L135" s="272" t="n"/>
       <c r="M135" s="273" t="n"/>
       <c r="N135" s="394">
-        <f>IF(C135&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O135" s="279" t="n"/>
@@ -15029,8 +15040,9 @@
       <c r="BM135" s="279" t="n"/>
       <c r="BN135" s="279" t="n"/>
       <c r="BO135" s="280" t="n"/>
-      <c r="BP135" s="394" t="n">
-        <v>0</v>
+      <c r="BP135" s="394">
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
+        <v/>
       </c>
       <c r="BQ135" s="279" t="n"/>
       <c r="BR135" s="279" t="n"/>
@@ -15048,11 +15060,12 @@
       <c r="CI135" s="316" t="n"/>
     </row>
     <row r="136" ht="15.75" customHeight="1" s="250">
-      <c r="C136" s="282" t="n">
-        <v>5</v>
+      <c r="C136" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D136" s="393">
-        <f>IF(C136&lt;=$I$15, EDATE($D$5, C136-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E136" s="272" t="n"/>
@@ -15065,7 +15078,7 @@
       <c r="L136" s="272" t="n"/>
       <c r="M136" s="273" t="n"/>
       <c r="N136" s="394">
-        <f>IF(C136&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O136" s="279" t="n"/>
@@ -15135,7 +15148,7 @@
       <c r="BN136" s="279" t="n"/>
       <c r="BO136" s="280" t="n"/>
       <c r="BP136" s="394">
-        <f>BP135</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ136" s="279" t="n"/>
@@ -15154,11 +15167,12 @@
       <c r="CI136" s="316" t="n"/>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="250">
-      <c r="C137" s="282" t="n">
-        <v>6</v>
+      <c r="C137" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D137" s="393">
-        <f>IF(C137&lt;=$I$15, EDATE($D$5, C137-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E137" s="272" t="n"/>
@@ -15171,7 +15185,7 @@
       <c r="L137" s="272" t="n"/>
       <c r="M137" s="273" t="n"/>
       <c r="N137" s="394">
-        <f>IF(C137&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O137" s="279" t="n"/>
@@ -15241,7 +15255,7 @@
       <c r="BN137" s="279" t="n"/>
       <c r="BO137" s="280" t="n"/>
       <c r="BP137" s="394">
-        <f>BP136</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ137" s="279" t="n"/>
@@ -15260,11 +15274,12 @@
       <c r="CI137" s="316" t="n"/>
     </row>
     <row r="138" ht="15.75" customHeight="1" s="250">
-      <c r="C138" s="282" t="n">
-        <v>7</v>
+      <c r="C138" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D138" s="393">
-        <f>IF(C138&lt;=$I$15, EDATE($D$5, C138-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E138" s="272" t="n"/>
@@ -15277,7 +15292,7 @@
       <c r="L138" s="272" t="n"/>
       <c r="M138" s="273" t="n"/>
       <c r="N138" s="394">
-        <f>IF(C138&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O138" s="279" t="n"/>
@@ -15347,7 +15362,7 @@
       <c r="BN138" s="279" t="n"/>
       <c r="BO138" s="280" t="n"/>
       <c r="BP138" s="394">
-        <f>BP137</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ138" s="279" t="n"/>
@@ -15366,11 +15381,12 @@
       <c r="CI138" s="316" t="n"/>
     </row>
     <row r="139" ht="15.75" customHeight="1" s="250">
-      <c r="C139" s="282" t="n">
-        <v>8</v>
+      <c r="C139" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D139" s="393">
-        <f>IF(C139&lt;=$I$15, EDATE($D$5, C139-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E139" s="272" t="n"/>
@@ -15383,7 +15399,7 @@
       <c r="L139" s="272" t="n"/>
       <c r="M139" s="273" t="n"/>
       <c r="N139" s="394">
-        <f>IF(C139&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O139" s="279" t="n"/>
@@ -15453,7 +15469,7 @@
       <c r="BN139" s="279" t="n"/>
       <c r="BO139" s="280" t="n"/>
       <c r="BP139" s="394">
-        <f>BP138</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ139" s="279" t="n"/>
@@ -15472,11 +15488,12 @@
       <c r="CI139" s="316" t="n"/>
     </row>
     <row r="140" ht="15.75" customHeight="1" s="250">
-      <c r="C140" s="282" t="n">
-        <v>9</v>
+      <c r="C140" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D140" s="393">
-        <f>IF(C140&lt;=$I$15, EDATE($D$5, C140-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E140" s="272" t="n"/>
@@ -15489,7 +15506,7 @@
       <c r="L140" s="272" t="n"/>
       <c r="M140" s="273" t="n"/>
       <c r="N140" s="394">
-        <f>IF(C140&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O140" s="279" t="n"/>
@@ -15559,7 +15576,7 @@
       <c r="BN140" s="279" t="n"/>
       <c r="BO140" s="280" t="n"/>
       <c r="BP140" s="394">
-        <f>BP139</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ140" s="279" t="n"/>
@@ -15578,11 +15595,12 @@
       <c r="CI140" s="316" t="n"/>
     </row>
     <row r="141" ht="15.75" customHeight="1" s="250">
-      <c r="C141" s="282" t="n">
-        <v>10</v>
+      <c r="C141" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D141" s="393">
-        <f>IF(C141&lt;=$I$15, EDATE($D$5, C141-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E141" s="272" t="n"/>
@@ -15595,7 +15613,7 @@
       <c r="L141" s="272" t="n"/>
       <c r="M141" s="273" t="n"/>
       <c r="N141" s="394">
-        <f>IF(C141&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O141" s="279" t="n"/>
@@ -15665,7 +15683,7 @@
       <c r="BN141" s="279" t="n"/>
       <c r="BO141" s="280" t="n"/>
       <c r="BP141" s="394">
-        <f>BP140</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ141" s="279" t="n"/>
@@ -15684,11 +15702,12 @@
       <c r="CI141" s="316" t="n"/>
     </row>
     <row r="142" ht="15.75" customHeight="1" s="250">
-      <c r="C142" s="282" t="n">
-        <v>11</v>
+      <c r="C142" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D142" s="393">
-        <f>IF(C142&lt;=$I$15, EDATE($D$5, C142-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E142" s="272" t="n"/>
@@ -15701,7 +15720,7 @@
       <c r="L142" s="272" t="n"/>
       <c r="M142" s="273" t="n"/>
       <c r="N142" s="394">
-        <f>IF(C142&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O142" s="279" t="n"/>
@@ -15770,8 +15789,9 @@
       <c r="BM142" s="279" t="n"/>
       <c r="BN142" s="279" t="n"/>
       <c r="BO142" s="280" t="n"/>
-      <c r="BP142" s="394" t="n">
-        <v>0</v>
+      <c r="BP142" s="394">
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
+        <v/>
       </c>
       <c r="BQ142" s="279" t="n"/>
       <c r="BR142" s="279" t="n"/>
@@ -15789,11 +15809,12 @@
       <c r="CI142" s="316" t="n"/>
     </row>
     <row r="143" ht="15.75" customHeight="1" s="250">
-      <c r="C143" s="282" t="n">
-        <v>12</v>
+      <c r="C143" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D143" s="393">
-        <f>IF(C143&lt;=$I$15, EDATE($D$5, C143-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E143" s="272" t="n"/>
@@ -15806,7 +15827,7 @@
       <c r="L143" s="272" t="n"/>
       <c r="M143" s="273" t="n"/>
       <c r="N143" s="394">
-        <f>IF(C143&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O143" s="279" t="n"/>
@@ -15875,8 +15896,9 @@
       <c r="BM143" s="279" t="n"/>
       <c r="BN143" s="279" t="n"/>
       <c r="BO143" s="280" t="n"/>
-      <c r="BP143" s="394" t="n">
-        <v>0</v>
+      <c r="BP143" s="394">
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
+        <v/>
       </c>
       <c r="BQ143" s="279" t="n"/>
       <c r="BR143" s="279" t="n"/>
@@ -15894,11 +15916,12 @@
       <c r="CI143" s="316" t="n"/>
     </row>
     <row r="144" ht="15.75" customHeight="1" s="250">
-      <c r="C144" s="282" t="n">
-        <v>13</v>
+      <c r="C144" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D144" s="393">
-        <f>IF(C144&lt;=$I$15, EDATE($D$5, C144-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E144" s="272" t="n"/>
@@ -15911,7 +15934,7 @@
       <c r="L144" s="272" t="n"/>
       <c r="M144" s="273" t="n"/>
       <c r="N144" s="394">
-        <f>IF(C144&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O144" s="279" t="n"/>
@@ -15980,8 +16003,9 @@
       <c r="BM144" s="279" t="n"/>
       <c r="BN144" s="279" t="n"/>
       <c r="BO144" s="280" t="n"/>
-      <c r="BP144" s="394" t="n">
-        <v>0</v>
+      <c r="BP144" s="394">
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
+        <v/>
       </c>
       <c r="BQ144" s="279" t="n"/>
       <c r="BR144" s="279" t="n"/>
@@ -15999,11 +16023,12 @@
       <c r="CI144" s="316" t="n"/>
     </row>
     <row r="145" ht="15.75" customHeight="1" s="250">
-      <c r="C145" s="282" t="n">
-        <v>14</v>
+      <c r="C145" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D145" s="393">
-        <f>IF(C145&lt;=$I$15, EDATE($D$5, C145-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E145" s="272" t="n"/>
@@ -16016,7 +16041,7 @@
       <c r="L145" s="272" t="n"/>
       <c r="M145" s="273" t="n"/>
       <c r="N145" s="394">
-        <f>IF(C145&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O145" s="279" t="n"/>
@@ -16086,7 +16111,7 @@
       <c r="BN145" s="279" t="n"/>
       <c r="BO145" s="280" t="n"/>
       <c r="BP145" s="394">
-        <f>BP144</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ145" s="279" t="n"/>
@@ -16105,11 +16130,12 @@
       <c r="CI145" s="316" t="n"/>
     </row>
     <row r="146" ht="15.75" customHeight="1" s="250">
-      <c r="C146" s="282" t="n">
-        <v>15</v>
+      <c r="C146" s="282">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D146" s="393">
-        <f>IF(C146&lt;=$I$15, EDATE($D$5, C146-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E146" s="272" t="n"/>
@@ -16122,7 +16148,7 @@
       <c r="L146" s="272" t="n"/>
       <c r="M146" s="273" t="n"/>
       <c r="N146" s="394">
-        <f>IF(C146&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O146" s="279" t="n"/>
@@ -16192,7 +16218,7 @@
       <c r="BN146" s="279" t="n"/>
       <c r="BO146" s="280" t="n"/>
       <c r="BP146" s="394">
-        <f>BP145</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ146" s="279" t="n"/>
@@ -16213,11 +16239,12 @@
     <row r="147" ht="15" customHeight="1" s="250">
       <c r="A147" s="396" t="n"/>
       <c r="B147" s="396" t="n"/>
-      <c r="C147" s="397" t="n">
-        <v>16</v>
+      <c r="C147" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D147" s="398">
-        <f>IF(C147&lt;=$I$15, EDATE($D$5, C147-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E147" s="272" t="n"/>
@@ -16230,7 +16257,7 @@
       <c r="L147" s="272" t="n"/>
       <c r="M147" s="273" t="n"/>
       <c r="N147" s="401">
-        <f>IF(C147&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O147" s="272" t="n"/>
@@ -16296,7 +16323,7 @@
       <c r="BN147" s="272" t="n"/>
       <c r="BO147" s="273" t="n"/>
       <c r="BP147" s="401">
-        <f>BP146</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ147" s="272" t="n"/>
@@ -16325,11 +16352,12 @@
     <row r="148" ht="15" customHeight="1" s="250">
       <c r="A148" s="396" t="n"/>
       <c r="B148" s="396" t="n"/>
-      <c r="C148" s="397" t="n">
-        <v>17</v>
+      <c r="C148" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D148" s="398">
-        <f>IF(C148&lt;=$I$15, EDATE($D$5, C148-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E148" s="272" t="n"/>
@@ -16342,7 +16370,7 @@
       <c r="L148" s="272" t="n"/>
       <c r="M148" s="273" t="n"/>
       <c r="N148" s="401">
-        <f>IF(C148&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O148" s="272" t="n"/>
@@ -16408,7 +16436,7 @@
       <c r="BN148" s="272" t="n"/>
       <c r="BO148" s="273" t="n"/>
       <c r="BP148" s="401">
-        <f>BP147</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ148" s="272" t="n"/>
@@ -16437,11 +16465,12 @@
     <row r="149" ht="15" customHeight="1" s="250">
       <c r="A149" s="396" t="n"/>
       <c r="B149" s="396" t="n"/>
-      <c r="C149" s="397" t="n">
-        <v>18</v>
+      <c r="C149" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D149" s="398">
-        <f>IF(C149&lt;=$I$15, EDATE($D$5, C149-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E149" s="272" t="n"/>
@@ -16454,7 +16483,7 @@
       <c r="L149" s="272" t="n"/>
       <c r="M149" s="273" t="n"/>
       <c r="N149" s="401">
-        <f>IF(C149&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O149" s="272" t="n"/>
@@ -16520,7 +16549,7 @@
       <c r="BN149" s="272" t="n"/>
       <c r="BO149" s="273" t="n"/>
       <c r="BP149" s="401">
-        <f>BP148</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ149" s="272" t="n"/>
@@ -16549,11 +16578,12 @@
     <row r="150" ht="15" customHeight="1" s="250">
       <c r="A150" s="396" t="n"/>
       <c r="B150" s="396" t="n"/>
-      <c r="C150" s="397" t="n">
-        <v>19</v>
+      <c r="C150" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D150" s="398">
-        <f>IF(C150&lt;=$I$15, EDATE($D$5, C150-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E150" s="272" t="n"/>
@@ -16566,7 +16596,7 @@
       <c r="L150" s="272" t="n"/>
       <c r="M150" s="273" t="n"/>
       <c r="N150" s="401">
-        <f>IF(C150&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O150" s="272" t="n"/>
@@ -16632,7 +16662,7 @@
       <c r="BN150" s="272" t="n"/>
       <c r="BO150" s="273" t="n"/>
       <c r="BP150" s="401">
-        <f>BP149</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ150" s="272" t="n"/>
@@ -16661,11 +16691,12 @@
     <row r="151" ht="15" customHeight="1" s="250">
       <c r="A151" s="396" t="n"/>
       <c r="B151" s="396" t="n"/>
-      <c r="C151" s="397" t="n">
-        <v>20</v>
+      <c r="C151" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D151" s="398">
-        <f>IF(C151&lt;=$I$15, EDATE($D$5, C151-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E151" s="272" t="n"/>
@@ -16678,7 +16709,7 @@
       <c r="L151" s="272" t="n"/>
       <c r="M151" s="273" t="n"/>
       <c r="N151" s="401">
-        <f>IF(C151&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O151" s="272" t="n"/>
@@ -16744,7 +16775,7 @@
       <c r="BN151" s="272" t="n"/>
       <c r="BO151" s="273" t="n"/>
       <c r="BP151" s="401">
-        <f>BP150</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ151" s="272" t="n"/>
@@ -16773,11 +16804,12 @@
     <row r="152" ht="15" customHeight="1" s="250">
       <c r="A152" s="396" t="n"/>
       <c r="B152" s="396" t="n"/>
-      <c r="C152" s="397" t="n">
-        <v>21</v>
+      <c r="C152" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D152" s="398">
-        <f>IF(C152&lt;=$I$15, EDATE($D$5, C152-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E152" s="272" t="n"/>
@@ -16790,7 +16822,7 @@
       <c r="L152" s="272" t="n"/>
       <c r="M152" s="273" t="n"/>
       <c r="N152" s="401">
-        <f>IF(C152&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O152" s="272" t="n"/>
@@ -16856,7 +16888,7 @@
       <c r="BN152" s="272" t="n"/>
       <c r="BO152" s="273" t="n"/>
       <c r="BP152" s="401">
-        <f>BP151</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ152" s="272" t="n"/>
@@ -16885,11 +16917,12 @@
     <row r="153" ht="15" customHeight="1" s="250">
       <c r="A153" s="396" t="n"/>
       <c r="B153" s="396" t="n"/>
-      <c r="C153" s="397" t="n">
-        <v>22</v>
+      <c r="C153" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D153" s="398">
-        <f>IF(C153&lt;=$I$15, EDATE($D$5, C153-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E153" s="272" t="n"/>
@@ -16902,7 +16935,7 @@
       <c r="L153" s="272" t="n"/>
       <c r="M153" s="273" t="n"/>
       <c r="N153" s="401">
-        <f>IF(C153&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O153" s="272" t="n"/>
@@ -16968,7 +17001,7 @@
       <c r="BN153" s="272" t="n"/>
       <c r="BO153" s="273" t="n"/>
       <c r="BP153" s="401">
-        <f>BP152</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ153" s="272" t="n"/>
@@ -16997,11 +17030,12 @@
     <row r="154" ht="12.75" customHeight="1" s="250">
       <c r="A154" s="396" t="n"/>
       <c r="B154" s="396" t="n"/>
-      <c r="C154" s="397" t="n">
-        <v>23</v>
+      <c r="C154" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D154" s="398">
-        <f>IF(C154&lt;=$I$15, EDATE($D$5, C154-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E154" s="272" t="n"/>
@@ -17014,7 +17048,7 @@
       <c r="L154" s="272" t="n"/>
       <c r="M154" s="273" t="n"/>
       <c r="N154" s="401">
-        <f>IF(C154&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O154" s="272" t="n"/>
@@ -17080,7 +17114,7 @@
       <c r="BN154" s="272" t="n"/>
       <c r="BO154" s="273" t="n"/>
       <c r="BP154" s="401">
-        <f>BP153</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ154" s="272" t="n"/>
@@ -17109,11 +17143,12 @@
     <row r="155" ht="12.75" customHeight="1" s="250">
       <c r="A155" s="396" t="n"/>
       <c r="B155" s="396" t="n"/>
-      <c r="C155" s="397" t="n">
-        <v>24</v>
+      <c r="C155" s="397">
+        <f>IF(ROW()-131&gt;$I$15,"",ROW()-131)</f>
+        <v/>
       </c>
       <c r="D155" s="398">
-        <f>IF(C155&lt;=$I$15, EDATE($D$5, C155-1), "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",EDATE($D$5,ROW()-132))</f>
         <v/>
       </c>
       <c r="E155" s="272" t="n"/>
@@ -17126,7 +17161,7 @@
       <c r="L155" s="272" t="n"/>
       <c r="M155" s="273" t="n"/>
       <c r="N155" s="401">
-        <f>IF(C155&lt;=$I$15, $I$16, "")</f>
+        <f>IF(ROW()-131&gt;$I$15,"",$I$16)</f>
         <v/>
       </c>
       <c r="O155" s="272" t="n"/>
@@ -17192,7 +17227,7 @@
       <c r="BN155" s="272" t="n"/>
       <c r="BO155" s="273" t="n"/>
       <c r="BP155" s="401">
-        <f>BP154</f>
+        <f>IF(ROW()-131&gt;$I$15,"",IF(ROW()-131&lt;=$BL$8,$I$16,""))</f>
         <v/>
       </c>
       <c r="BQ155" s="272" t="n"/>
@@ -17246,9 +17281,9 @@
   <mergeCells count="382">
     <mergeCell ref="I9:Y9"/>
     <mergeCell ref="BE17:BK17"/>
+    <mergeCell ref="AE148:AN148"/>
+    <mergeCell ref="N148:Y148"/>
     <mergeCell ref="D133:M133"/>
-    <mergeCell ref="N148:Y148"/>
-    <mergeCell ref="AE148:AN148"/>
     <mergeCell ref="I11:Y11"/>
     <mergeCell ref="BE19:BK19"/>
     <mergeCell ref="BF142:BO142"/>

</xml_diff>